<commit_message>
📊 Update NAIC content history - 2026-08-25
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5AC089-19A3-420E-8B06-D330B0BC2D2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32422558-6F26-48C4-B42A-A869249C86BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45090" yWindow="3105" windowWidth="18720" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -679,6 +679,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Notes"/>
@@ -7867,51 +7868,51 @@
           <cell r="H238">
             <v>46256</v>
           </cell>
-          <cell r="I238" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J238" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K238" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L238" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I238">
+            <v>4.6300000000000001E-2</v>
+          </cell>
+          <cell r="J238">
+            <v>4.9399999999999999E-2</v>
+          </cell>
+          <cell r="K238">
+            <v>5.1799999999999999E-2</v>
+          </cell>
+          <cell r="L238">
+            <v>5.4399999999999997E-2</v>
           </cell>
         </row>
         <row r="239">
           <cell r="H239">
             <v>46257</v>
           </cell>
-          <cell r="I239" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J239" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K239" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L239" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I239">
+            <v>4.6300000000000001E-2</v>
+          </cell>
+          <cell r="J239">
+            <v>4.9399999999999999E-2</v>
+          </cell>
+          <cell r="K239">
+            <v>5.1799999999999999E-2</v>
+          </cell>
+          <cell r="L239">
+            <v>5.4399999999999997E-2</v>
           </cell>
         </row>
         <row r="240">
           <cell r="H240">
             <v>46258</v>
           </cell>
-          <cell r="I240" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J240" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K240" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L240" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I240">
+            <v>4.6300000000000001E-2</v>
+          </cell>
+          <cell r="J240">
+            <v>4.9399999999999999E-2</v>
+          </cell>
+          <cell r="K240">
+            <v>5.1799999999999999E-2</v>
+          </cell>
+          <cell r="L240">
+            <v>5.4399999999999997E-2</v>
           </cell>
         </row>
         <row r="241">
@@ -10131,9 +10132,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -10171,9 +10172,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -10206,26 +10207,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -10258,26 +10242,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -15648,21 +15615,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
       </c>
-      <c r="B237" s="17" t="str">
+      <c r="B237" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I238</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C237" s="47" t="str">
+        <v>4.6300000000000001E-2</v>
+      </c>
+      <c r="C237" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J238</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D237" s="47" t="str">
+        <v>4.9399999999999999E-2</v>
+      </c>
+      <c r="D237" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K238</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E237" s="5" t="str">
+        <v>5.1799999999999999E-2</v>
+      </c>
+      <c r="E237" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L238</f>
-        <v xml:space="preserve"> </v>
+        <v>5.4399999999999997E-2</v>
       </c>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.35">
@@ -15670,21 +15637,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
       </c>
-      <c r="B238" s="17" t="str">
+      <c r="B238" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I239</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C238" s="47" t="str">
+        <v>4.6300000000000001E-2</v>
+      </c>
+      <c r="C238" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J239</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D238" s="47" t="str">
+        <v>4.9399999999999999E-2</v>
+      </c>
+      <c r="D238" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K239</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E238" s="5" t="str">
+        <v>5.1799999999999999E-2</v>
+      </c>
+      <c r="E238" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L239</f>
-        <v xml:space="preserve"> </v>
+        <v>5.4399999999999997E-2</v>
       </c>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.35">
@@ -15692,21 +15659,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
       </c>
-      <c r="B239" s="17" t="str">
+      <c r="B239" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I240</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C239" s="47" t="str">
+        <v>4.6300000000000001E-2</v>
+      </c>
+      <c r="C239" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J240</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D239" s="47" t="str">
+        <v>4.9399999999999999E-2</v>
+      </c>
+      <c r="D239" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K240</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E239" s="5" t="str">
+        <v>5.1799999999999999E-2</v>
+      </c>
+      <c r="E239" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L240</f>
-        <v xml:space="preserve"> </v>
+        <v>5.4399999999999997E-2</v>
       </c>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.35">
@@ -19422,182 +19389,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="str" cm="1">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="str">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
@@ -25299,18 +25266,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>